<commit_message>
updated age groups files
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/agegroups/DE-AgeGroups_de.xlsx
+++ b/owlcms/src/main/resources/agegroups/DE-AgeGroups_de.xlsx
@@ -685,8 +685,8 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="J2" s="2" t="s">
-        <v>11</v>
+      <c r="J2" s="2">
+        <v>999</v>
       </c>
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
@@ -728,27 +728,29 @@
       <c r="H3" t="s">
         <v>80</v>
       </c>
-      <c r="J3" s="2"/>
-      <c r="K3" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="L3" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="M3" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="N3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="O3" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="P3" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="Q3" s="2" t="s">
-        <v>11</v>
+      <c r="J3" s="2">
+        <v>40</v>
+      </c>
+      <c r="K3" s="2">
+        <v>44</v>
+      </c>
+      <c r="L3" s="2">
+        <v>45</v>
+      </c>
+      <c r="M3" s="2">
+        <v>49</v>
+      </c>
+      <c r="N3" s="2">
+        <v>53</v>
+      </c>
+      <c r="O3" s="2">
+        <v>57</v>
+      </c>
+      <c r="P3" s="2">
+        <v>61</v>
+      </c>
+      <c r="Q3" s="2">
+        <v>999</v>
       </c>
       <c r="R3" s="2"/>
       <c r="S3" s="2"/>
@@ -783,27 +785,29 @@
       <c r="H4" t="s">
         <v>80</v>
       </c>
-      <c r="J4" s="2"/>
-      <c r="K4" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="L4" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="M4" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="N4" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="O4" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="P4" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="Q4" s="2" t="s">
-        <v>11</v>
+      <c r="J4" s="2">
+        <v>40</v>
+      </c>
+      <c r="K4" s="2">
+        <v>44</v>
+      </c>
+      <c r="L4" s="2">
+        <v>45</v>
+      </c>
+      <c r="M4" s="2">
+        <v>49</v>
+      </c>
+      <c r="N4" s="2">
+        <v>53</v>
+      </c>
+      <c r="O4" s="2">
+        <v>57</v>
+      </c>
+      <c r="P4" s="2">
+        <v>61</v>
+      </c>
+      <c r="Q4" s="2">
+        <v>999</v>
       </c>
       <c r="R4" s="2"/>
       <c r="S4" s="2"/>
@@ -838,32 +842,32 @@
       <c r="H5" t="s">
         <v>80</v>
       </c>
-      <c r="J5" s="2"/>
-      <c r="K5" s="2"/>
-      <c r="L5" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="M5" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="N5" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="O5" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="P5" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="Q5" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="R5" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="S5" s="2" t="s">
-        <v>11</v>
-      </c>
+      <c r="J5" s="2">
+        <v>45</v>
+      </c>
+      <c r="K5" s="2">
+        <v>49</v>
+      </c>
+      <c r="L5" s="2">
+        <v>53</v>
+      </c>
+      <c r="M5" s="2">
+        <v>57</v>
+      </c>
+      <c r="N5" s="2">
+        <v>61</v>
+      </c>
+      <c r="O5" s="2">
+        <v>69</v>
+      </c>
+      <c r="P5" s="2">
+        <v>77</v>
+      </c>
+      <c r="Q5" s="2">
+        <v>999</v>
+      </c>
+      <c r="R5" s="2"/>
+      <c r="S5" s="2"/>
       <c r="T5" s="2"/>
       <c r="U5" s="2"/>
       <c r="V5" s="2"/>
@@ -895,40 +899,34 @@
       <c r="H6" t="s">
         <v>80</v>
       </c>
-      <c r="J6" s="2"/>
-      <c r="K6" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="L6" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="M6" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="N6" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="O6" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="P6" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q6" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="R6" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="S6" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="T6" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="U6" s="2" t="s">
-        <v>11</v>
-      </c>
+      <c r="J6" s="2">
+        <v>49</v>
+      </c>
+      <c r="K6" s="2">
+        <v>53</v>
+      </c>
+      <c r="L6" s="2">
+        <v>57</v>
+      </c>
+      <c r="M6" s="2">
+        <v>61</v>
+      </c>
+      <c r="N6" s="2">
+        <v>69</v>
+      </c>
+      <c r="O6" s="2">
+        <v>77</v>
+      </c>
+      <c r="P6" s="2">
+        <v>86</v>
+      </c>
+      <c r="Q6" s="2">
+        <v>999</v>
+      </c>
+      <c r="R6" s="2"/>
+      <c r="S6" s="2"/>
+      <c r="T6" s="2"/>
+      <c r="U6" s="2"/>
       <c r="V6" s="2"/>
       <c r="W6" s="2"/>
     </row>
@@ -958,40 +956,34 @@
       <c r="H7" t="s">
         <v>80</v>
       </c>
-      <c r="J7" s="2"/>
-      <c r="K7" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="L7" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="M7" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="N7" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="O7" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="P7" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q7" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="R7" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="S7" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="T7" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="U7" s="2" t="s">
-        <v>11</v>
-      </c>
+      <c r="J7" s="2">
+        <v>49</v>
+      </c>
+      <c r="K7" s="2">
+        <v>53</v>
+      </c>
+      <c r="L7" s="2">
+        <v>57</v>
+      </c>
+      <c r="M7" s="2">
+        <v>61</v>
+      </c>
+      <c r="N7" s="2">
+        <v>69</v>
+      </c>
+      <c r="O7" s="2">
+        <v>77</v>
+      </c>
+      <c r="P7" s="2">
+        <v>86</v>
+      </c>
+      <c r="Q7" s="2">
+        <v>999</v>
+      </c>
+      <c r="R7" s="2"/>
+      <c r="S7" s="2"/>
+      <c r="T7" s="2"/>
+      <c r="U7" s="2"/>
       <c r="V7" s="2"/>
       <c r="W7" s="2"/>
     </row>
@@ -1021,40 +1013,34 @@
       <c r="H8" t="s">
         <v>80</v>
       </c>
-      <c r="J8" s="2"/>
-      <c r="K8" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="L8" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="M8" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="N8" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="O8" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="P8" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q8" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="R8" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="S8" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="T8" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="U8" s="2" t="s">
-        <v>11</v>
-      </c>
+      <c r="J8" s="2">
+        <v>49</v>
+      </c>
+      <c r="K8" s="2">
+        <v>53</v>
+      </c>
+      <c r="L8" s="2">
+        <v>57</v>
+      </c>
+      <c r="M8" s="2">
+        <v>61</v>
+      </c>
+      <c r="N8" s="2">
+        <v>69</v>
+      </c>
+      <c r="O8" s="2">
+        <v>77</v>
+      </c>
+      <c r="P8" s="2">
+        <v>86</v>
+      </c>
+      <c r="Q8" s="2">
+        <v>999</v>
+      </c>
+      <c r="R8" s="2"/>
+      <c r="S8" s="2"/>
+      <c r="T8" s="2"/>
+      <c r="U8" s="2"/>
       <c r="V8" s="2"/>
       <c r="W8" s="2"/>
     </row>
@@ -1084,40 +1070,34 @@
       <c r="H9" t="s">
         <v>80</v>
       </c>
-      <c r="J9" s="2"/>
-      <c r="K9" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="L9" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="M9" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="N9" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="O9" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="P9" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q9" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="R9" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="S9" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="T9" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="U9" s="2" t="s">
-        <v>11</v>
-      </c>
+      <c r="J9" s="2">
+        <v>49</v>
+      </c>
+      <c r="K9" s="2">
+        <v>53</v>
+      </c>
+      <c r="L9" s="2">
+        <v>57</v>
+      </c>
+      <c r="M9" s="2">
+        <v>61</v>
+      </c>
+      <c r="N9" s="2">
+        <v>69</v>
+      </c>
+      <c r="O9" s="2">
+        <v>77</v>
+      </c>
+      <c r="P9" s="2">
+        <v>86</v>
+      </c>
+      <c r="Q9" s="2">
+        <v>999</v>
+      </c>
+      <c r="R9" s="2"/>
+      <c r="S9" s="2"/>
+      <c r="T9" s="2"/>
+      <c r="U9" s="2"/>
       <c r="V9" s="2"/>
       <c r="W9" s="2"/>
     </row>
@@ -1144,40 +1124,34 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="J10" s="2"/>
-      <c r="K10" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="L10" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="M10" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="N10" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="O10" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="P10" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q10" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="R10" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="S10" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="T10" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="U10" s="2" t="s">
-        <v>11</v>
-      </c>
+      <c r="J10" s="2">
+        <v>49</v>
+      </c>
+      <c r="K10" s="2">
+        <v>53</v>
+      </c>
+      <c r="L10" s="2">
+        <v>57</v>
+      </c>
+      <c r="M10" s="2">
+        <v>61</v>
+      </c>
+      <c r="N10" s="2">
+        <v>69</v>
+      </c>
+      <c r="O10" s="2">
+        <v>77</v>
+      </c>
+      <c r="P10" s="2">
+        <v>86</v>
+      </c>
+      <c r="Q10" s="2">
+        <v>999</v>
+      </c>
+      <c r="R10" s="2"/>
+      <c r="S10" s="2"/>
+      <c r="T10" s="2"/>
+      <c r="U10" s="2"/>
       <c r="V10" s="2"/>
       <c r="W10" s="2"/>
     </row>
@@ -1204,40 +1178,34 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="J11" s="2"/>
-      <c r="K11" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="L11" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="M11" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="N11" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="O11" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="P11" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q11" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="R11" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="S11" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="T11" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="U11" s="2" t="s">
-        <v>11</v>
-      </c>
+      <c r="J11" s="2">
+        <v>49</v>
+      </c>
+      <c r="K11" s="2">
+        <v>53</v>
+      </c>
+      <c r="L11" s="2">
+        <v>57</v>
+      </c>
+      <c r="M11" s="2">
+        <v>61</v>
+      </c>
+      <c r="N11" s="2">
+        <v>69</v>
+      </c>
+      <c r="O11" s="2">
+        <v>77</v>
+      </c>
+      <c r="P11" s="2">
+        <v>86</v>
+      </c>
+      <c r="Q11" s="2">
+        <v>999</v>
+      </c>
+      <c r="R11" s="2"/>
+      <c r="S11" s="2"/>
+      <c r="T11" s="2"/>
+      <c r="U11" s="2"/>
       <c r="V11" s="2"/>
       <c r="W11" s="2"/>
     </row>
@@ -1267,40 +1235,34 @@
       <c r="H12" t="s">
         <v>80</v>
       </c>
-      <c r="J12" s="2"/>
-      <c r="K12" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="L12" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="M12" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="N12" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="O12" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="P12" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q12" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="R12" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="S12" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="T12" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="U12" s="2" t="s">
-        <v>11</v>
-      </c>
+      <c r="J12" s="2">
+        <v>49</v>
+      </c>
+      <c r="K12" s="2">
+        <v>53</v>
+      </c>
+      <c r="L12" s="2">
+        <v>57</v>
+      </c>
+      <c r="M12" s="2">
+        <v>61</v>
+      </c>
+      <c r="N12" s="2">
+        <v>69</v>
+      </c>
+      <c r="O12" s="2">
+        <v>77</v>
+      </c>
+      <c r="P12" s="2">
+        <v>86</v>
+      </c>
+      <c r="Q12" s="2">
+        <v>999</v>
+      </c>
+      <c r="R12" s="2"/>
+      <c r="S12" s="2"/>
+      <c r="T12" s="2"/>
+      <c r="U12" s="2"/>
       <c r="V12" s="2"/>
       <c r="W12" s="2"/>
     </row>
@@ -1330,40 +1292,34 @@
       <c r="H13" t="s">
         <v>80</v>
       </c>
-      <c r="J13" s="2"/>
-      <c r="K13" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="L13" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="M13" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="N13" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="O13" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="P13" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q13" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="R13" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="S13" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="T13" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="U13" s="2" t="s">
-        <v>11</v>
-      </c>
+      <c r="J13" s="2">
+        <v>49</v>
+      </c>
+      <c r="K13" s="2">
+        <v>53</v>
+      </c>
+      <c r="L13" s="2">
+        <v>57</v>
+      </c>
+      <c r="M13" s="2">
+        <v>61</v>
+      </c>
+      <c r="N13" s="2">
+        <v>69</v>
+      </c>
+      <c r="O13" s="2">
+        <v>77</v>
+      </c>
+      <c r="P13" s="2">
+        <v>86</v>
+      </c>
+      <c r="Q13" s="2">
+        <v>999</v>
+      </c>
+      <c r="R13" s="2"/>
+      <c r="S13" s="2"/>
+      <c r="T13" s="2"/>
+      <c r="U13" s="2"/>
       <c r="V13" s="2"/>
       <c r="W13" s="2"/>
     </row>
@@ -1393,40 +1349,34 @@
       <c r="H14" t="s">
         <v>80</v>
       </c>
-      <c r="J14" s="2"/>
-      <c r="K14" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="L14" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="M14" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="N14" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="O14" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="P14" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q14" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="R14" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="S14" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="T14" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="U14" s="2" t="s">
-        <v>11</v>
-      </c>
+      <c r="J14" s="2">
+        <v>49</v>
+      </c>
+      <c r="K14" s="2">
+        <v>53</v>
+      </c>
+      <c r="L14" s="2">
+        <v>57</v>
+      </c>
+      <c r="M14" s="2">
+        <v>61</v>
+      </c>
+      <c r="N14" s="2">
+        <v>69</v>
+      </c>
+      <c r="O14" s="2">
+        <v>77</v>
+      </c>
+      <c r="P14" s="2">
+        <v>86</v>
+      </c>
+      <c r="Q14" s="2">
+        <v>999</v>
+      </c>
+      <c r="R14" s="2"/>
+      <c r="S14" s="2"/>
+      <c r="T14" s="2"/>
+      <c r="U14" s="2"/>
       <c r="V14" s="2"/>
       <c r="W14" s="2"/>
     </row>
@@ -1456,40 +1406,34 @@
       <c r="H15" t="s">
         <v>80</v>
       </c>
-      <c r="J15" s="2"/>
-      <c r="K15" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="L15" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="M15" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="N15" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="O15" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="P15" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q15" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="R15" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="S15" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="T15" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="U15" s="2" t="s">
-        <v>11</v>
-      </c>
+      <c r="J15" s="2">
+        <v>49</v>
+      </c>
+      <c r="K15" s="2">
+        <v>53</v>
+      </c>
+      <c r="L15" s="2">
+        <v>57</v>
+      </c>
+      <c r="M15" s="2">
+        <v>61</v>
+      </c>
+      <c r="N15" s="2">
+        <v>69</v>
+      </c>
+      <c r="O15" s="2">
+        <v>77</v>
+      </c>
+      <c r="P15" s="2">
+        <v>86</v>
+      </c>
+      <c r="Q15" s="2">
+        <v>999</v>
+      </c>
+      <c r="R15" s="2"/>
+      <c r="S15" s="2"/>
+      <c r="T15" s="2"/>
+      <c r="U15" s="2"/>
       <c r="V15" s="2"/>
       <c r="W15" s="2"/>
     </row>
@@ -1519,40 +1463,34 @@
       <c r="H16" t="s">
         <v>80</v>
       </c>
-      <c r="J16" s="2"/>
-      <c r="K16" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="L16" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="M16" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="N16" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="O16" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="P16" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q16" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="R16" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="S16" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="T16" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="U16" s="2" t="s">
-        <v>11</v>
-      </c>
+      <c r="J16" s="2">
+        <v>49</v>
+      </c>
+      <c r="K16" s="2">
+        <v>53</v>
+      </c>
+      <c r="L16" s="2">
+        <v>57</v>
+      </c>
+      <c r="M16" s="2">
+        <v>61</v>
+      </c>
+      <c r="N16" s="2">
+        <v>69</v>
+      </c>
+      <c r="O16" s="2">
+        <v>77</v>
+      </c>
+      <c r="P16" s="2">
+        <v>86</v>
+      </c>
+      <c r="Q16" s="2">
+        <v>999</v>
+      </c>
+      <c r="R16" s="2"/>
+      <c r="S16" s="2"/>
+      <c r="T16" s="2"/>
+      <c r="U16" s="2"/>
       <c r="V16" s="2"/>
       <c r="W16" s="2"/>
     </row>
@@ -1582,40 +1520,34 @@
       <c r="H17" t="s">
         <v>80</v>
       </c>
-      <c r="J17" s="2"/>
-      <c r="K17" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="L17" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="M17" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="N17" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="O17" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="P17" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q17" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="R17" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="S17" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="T17" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="U17" s="2" t="s">
-        <v>11</v>
-      </c>
+      <c r="J17" s="2">
+        <v>49</v>
+      </c>
+      <c r="K17" s="2">
+        <v>53</v>
+      </c>
+      <c r="L17" s="2">
+        <v>57</v>
+      </c>
+      <c r="M17" s="2">
+        <v>61</v>
+      </c>
+      <c r="N17" s="2">
+        <v>69</v>
+      </c>
+      <c r="O17" s="2">
+        <v>77</v>
+      </c>
+      <c r="P17" s="2">
+        <v>86</v>
+      </c>
+      <c r="Q17" s="2">
+        <v>999</v>
+      </c>
+      <c r="R17" s="2"/>
+      <c r="S17" s="2"/>
+      <c r="T17" s="2"/>
+      <c r="U17" s="2"/>
       <c r="V17" s="2"/>
       <c r="W17" s="2"/>
     </row>
@@ -1645,40 +1577,34 @@
       <c r="H18" t="s">
         <v>80</v>
       </c>
-      <c r="J18" s="2"/>
-      <c r="K18" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="L18" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="M18" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="N18" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="O18" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="P18" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q18" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="R18" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="S18" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="T18" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="U18" s="2" t="s">
-        <v>11</v>
-      </c>
+      <c r="J18" s="2">
+        <v>49</v>
+      </c>
+      <c r="K18" s="2">
+        <v>53</v>
+      </c>
+      <c r="L18" s="2">
+        <v>57</v>
+      </c>
+      <c r="M18" s="2">
+        <v>61</v>
+      </c>
+      <c r="N18" s="2">
+        <v>69</v>
+      </c>
+      <c r="O18" s="2">
+        <v>77</v>
+      </c>
+      <c r="P18" s="2">
+        <v>86</v>
+      </c>
+      <c r="Q18" s="2">
+        <v>999</v>
+      </c>
+      <c r="R18" s="2"/>
+      <c r="S18" s="2"/>
+      <c r="T18" s="2"/>
+      <c r="U18" s="2"/>
       <c r="V18" s="2"/>
       <c r="W18" s="2"/>
     </row>
@@ -1708,40 +1634,34 @@
       <c r="H19" t="s">
         <v>80</v>
       </c>
-      <c r="J19" s="2"/>
-      <c r="K19" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="L19" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="M19" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="N19" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="O19" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="P19" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q19" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="R19" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="S19" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="T19" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="U19" s="2" t="s">
-        <v>11</v>
-      </c>
+      <c r="J19" s="2">
+        <v>49</v>
+      </c>
+      <c r="K19" s="2">
+        <v>53</v>
+      </c>
+      <c r="L19" s="2">
+        <v>57</v>
+      </c>
+      <c r="M19" s="2">
+        <v>61</v>
+      </c>
+      <c r="N19" s="2">
+        <v>69</v>
+      </c>
+      <c r="O19" s="2">
+        <v>77</v>
+      </c>
+      <c r="P19" s="2">
+        <v>86</v>
+      </c>
+      <c r="Q19" s="2">
+        <v>999</v>
+      </c>
+      <c r="R19" s="2"/>
+      <c r="S19" s="2"/>
+      <c r="T19" s="2"/>
+      <c r="U19" s="2"/>
       <c r="V19" s="2"/>
       <c r="W19" s="2"/>
     </row>
@@ -1771,40 +1691,34 @@
       <c r="H20" t="s">
         <v>80</v>
       </c>
-      <c r="J20" s="2"/>
-      <c r="K20" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="L20" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="M20" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="N20" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="O20" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="P20" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q20" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="R20" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="S20" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="T20" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="U20" s="2" t="s">
-        <v>11</v>
-      </c>
+      <c r="J20" s="2">
+        <v>49</v>
+      </c>
+      <c r="K20" s="2">
+        <v>53</v>
+      </c>
+      <c r="L20" s="2">
+        <v>57</v>
+      </c>
+      <c r="M20" s="2">
+        <v>61</v>
+      </c>
+      <c r="N20" s="2">
+        <v>69</v>
+      </c>
+      <c r="O20" s="2">
+        <v>77</v>
+      </c>
+      <c r="P20" s="2">
+        <v>86</v>
+      </c>
+      <c r="Q20" s="2">
+        <v>999</v>
+      </c>
+      <c r="R20" s="2"/>
+      <c r="S20" s="2"/>
+      <c r="T20" s="2"/>
+      <c r="U20" s="2"/>
       <c r="V20" s="2"/>
       <c r="W20" s="2"/>
     </row>
@@ -1834,37 +1748,33 @@
       <c r="H21" t="s">
         <v>80</v>
       </c>
-      <c r="J21" s="2"/>
-      <c r="K21" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="L21" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="M21" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="N21" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="O21" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="P21" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q21" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="R21" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="S21" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="T21" s="2" t="s">
-        <v>11</v>
-      </c>
+      <c r="J21" s="2">
+        <v>45</v>
+      </c>
+      <c r="K21" s="2">
+        <v>49</v>
+      </c>
+      <c r="L21" s="2">
+        <v>53</v>
+      </c>
+      <c r="M21" s="2">
+        <v>57</v>
+      </c>
+      <c r="N21" s="2">
+        <v>61</v>
+      </c>
+      <c r="O21" s="2">
+        <v>69</v>
+      </c>
+      <c r="P21" s="2">
+        <v>77</v>
+      </c>
+      <c r="Q21" s="2">
+        <v>999</v>
+      </c>
+      <c r="R21" s="2"/>
+      <c r="S21" s="2"/>
+      <c r="T21" s="2"/>
       <c r="U21" s="2"/>
       <c r="V21" s="2"/>
       <c r="W21" s="2"/>
@@ -1895,38 +1805,34 @@
       <c r="H22" t="s">
         <v>80</v>
       </c>
-      <c r="J22" s="2"/>
-      <c r="K22" s="2"/>
-      <c r="L22" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="M22" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="N22" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="O22" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="P22" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q22" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="R22" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="S22" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="T22" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="U22" s="2" t="s">
-        <v>11</v>
-      </c>
+      <c r="J22" s="2">
+        <v>49</v>
+      </c>
+      <c r="K22" s="2">
+        <v>53</v>
+      </c>
+      <c r="L22" s="2">
+        <v>57</v>
+      </c>
+      <c r="M22" s="2">
+        <v>61</v>
+      </c>
+      <c r="N22" s="2">
+        <v>69</v>
+      </c>
+      <c r="O22" s="2">
+        <v>77</v>
+      </c>
+      <c r="P22" s="2">
+        <v>86</v>
+      </c>
+      <c r="Q22" s="2">
+        <v>999</v>
+      </c>
+      <c r="R22" s="2"/>
+      <c r="S22" s="2"/>
+      <c r="T22" s="2"/>
+      <c r="U22" s="2"/>
       <c r="V22" s="2"/>
       <c r="W22" s="2"/>
     </row>
@@ -1956,38 +1862,34 @@
       <c r="H23" t="s">
         <v>80</v>
       </c>
-      <c r="J23" s="2"/>
-      <c r="K23" s="2"/>
-      <c r="L23" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="M23" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="N23" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="O23" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="P23" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q23" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="R23" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="S23" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="T23" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="U23" s="2" t="s">
-        <v>11</v>
-      </c>
+      <c r="J23" s="2">
+        <v>49</v>
+      </c>
+      <c r="K23" s="2">
+        <v>53</v>
+      </c>
+      <c r="L23" s="2">
+        <v>57</v>
+      </c>
+      <c r="M23" s="2">
+        <v>61</v>
+      </c>
+      <c r="N23" s="2">
+        <v>69</v>
+      </c>
+      <c r="O23" s="2">
+        <v>77</v>
+      </c>
+      <c r="P23" s="2">
+        <v>86</v>
+      </c>
+      <c r="Q23" s="2">
+        <v>999</v>
+      </c>
+      <c r="R23" s="2"/>
+      <c r="S23" s="2"/>
+      <c r="T23" s="2"/>
+      <c r="U23" s="2"/>
       <c r="V23" s="2"/>
       <c r="W23" s="2"/>
     </row>
@@ -2017,42 +1919,40 @@
       <c r="H24" t="s">
         <v>80</v>
       </c>
-      <c r="J24" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="K24" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="L24" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="M24" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="N24" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="O24" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="P24" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q24" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="R24" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="S24" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="T24" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="U24" s="2" t="s">
-        <v>11</v>
-      </c>
+      <c r="J24" s="2">
+        <v>40</v>
+      </c>
+      <c r="K24" s="2">
+        <v>44</v>
+      </c>
+      <c r="L24" s="2">
+        <v>45</v>
+      </c>
+      <c r="M24" s="2">
+        <v>49</v>
+      </c>
+      <c r="N24" s="2">
+        <v>53</v>
+      </c>
+      <c r="O24" s="2">
+        <v>57</v>
+      </c>
+      <c r="P24" s="2">
+        <v>61</v>
+      </c>
+      <c r="Q24" s="2">
+        <v>69</v>
+      </c>
+      <c r="R24" s="2">
+        <v>77</v>
+      </c>
+      <c r="S24" s="2">
+        <v>86</v>
+      </c>
+      <c r="T24" s="2">
+        <v>999</v>
+      </c>
+      <c r="U24" s="2"/>
       <c r="V24" s="2"/>
       <c r="W24" s="2"/>
     </row>
@@ -2079,8 +1979,8 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="J25" s="2" t="s">
-        <v>51</v>
+      <c r="J25" s="2">
+        <v>999</v>
       </c>
       <c r="K25" s="2"/>
       <c r="L25" s="2"/>
@@ -2122,29 +2022,29 @@
       <c r="H26" t="s">
         <v>80</v>
       </c>
-      <c r="J26" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="K26" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="L26" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="M26" s="2" t="s">
+      <c r="J26" s="2">
+        <v>35</v>
+      </c>
+      <c r="K26" s="2">
+        <v>40</v>
+      </c>
+      <c r="L26" s="2">
+        <v>45</v>
+      </c>
+      <c r="M26" s="2">
+        <v>50</v>
+      </c>
+      <c r="N26" s="2">
         <v>55</v>
       </c>
-      <c r="N26" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="O26" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="P26" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q26" s="2" t="s">
-        <v>51</v>
+      <c r="O26" s="2">
+        <v>60</v>
+      </c>
+      <c r="P26" s="2">
+        <v>65</v>
+      </c>
+      <c r="Q26" s="2">
+        <v>999</v>
       </c>
       <c r="R26" s="2"/>
       <c r="S26" s="2"/>
@@ -2179,34 +2079,32 @@
       <c r="H27" t="s">
         <v>80</v>
       </c>
-      <c r="J27" s="2"/>
-      <c r="K27" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="L27" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="M27" s="2" t="s">
+      <c r="J27" s="2">
+        <v>40</v>
+      </c>
+      <c r="K27" s="2">
+        <v>45</v>
+      </c>
+      <c r="L27" s="2">
+        <v>50</v>
+      </c>
+      <c r="M27" s="2">
         <v>55</v>
       </c>
-      <c r="N27" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="O27" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="P27" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q27" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="R27" s="2" t="s">
+      <c r="N27" s="2">
         <v>60</v>
       </c>
-      <c r="S27" s="2" t="s">
-        <v>51</v>
-      </c>
+      <c r="O27" s="2">
+        <v>65</v>
+      </c>
+      <c r="P27" s="2">
+        <v>70</v>
+      </c>
+      <c r="Q27" s="2">
+        <v>999</v>
+      </c>
+      <c r="R27" s="2"/>
+      <c r="S27" s="2"/>
       <c r="T27" s="2"/>
       <c r="U27" s="2"/>
       <c r="V27" s="2"/>
@@ -2238,33 +2136,33 @@
       <c r="H28" t="s">
         <v>80</v>
       </c>
-      <c r="J28" s="2"/>
-      <c r="K28" s="2"/>
-      <c r="L28" s="2"/>
-      <c r="M28" s="2" t="s">
+      <c r="J28" s="2">
         <v>55</v>
       </c>
-      <c r="N28" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="O28" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="P28" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q28" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="R28" s="2" t="s">
+      <c r="K28" s="2">
         <v>60</v>
       </c>
-      <c r="S28" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="T28" s="2" t="s">
-        <v>51</v>
-      </c>
+      <c r="L28" s="2">
+        <v>65</v>
+      </c>
+      <c r="M28" s="2">
+        <v>70</v>
+      </c>
+      <c r="N28" s="2">
+        <v>75</v>
+      </c>
+      <c r="O28" s="2">
+        <v>85</v>
+      </c>
+      <c r="P28" s="2">
+        <v>95</v>
+      </c>
+      <c r="Q28" s="2">
+        <v>999</v>
+      </c>
+      <c r="R28" s="2"/>
+      <c r="S28" s="2"/>
+      <c r="T28" s="2"/>
       <c r="U28" s="2"/>
       <c r="V28" s="2"/>
       <c r="W28" s="2"/>
@@ -2295,40 +2193,36 @@
       <c r="H29" t="s">
         <v>80</v>
       </c>
-      <c r="J29" s="2"/>
-      <c r="K29" s="2"/>
-      <c r="L29" s="2"/>
-      <c r="M29" s="2"/>
-      <c r="N29" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="O29" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="P29" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="Q29" s="2" t="s">
+      <c r="J29" s="2">
+        <v>60</v>
+      </c>
+      <c r="K29" s="2">
         <v>65</v>
       </c>
-      <c r="R29" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="S29" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="T29" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="U29" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="V29" s="2" t="s">
+      <c r="L29" s="2">
         <v>70</v>
       </c>
-      <c r="W29" s="2" t="s">
-        <v>51</v>
-      </c>
+      <c r="M29" s="2">
+        <v>75</v>
+      </c>
+      <c r="N29" s="2">
+        <v>85</v>
+      </c>
+      <c r="O29" s="2">
+        <v>95</v>
+      </c>
+      <c r="P29" s="2">
+        <v>110</v>
+      </c>
+      <c r="Q29" s="2">
+        <v>999</v>
+      </c>
+      <c r="R29" s="2"/>
+      <c r="S29" s="2"/>
+      <c r="T29" s="2"/>
+      <c r="U29" s="2"/>
+      <c r="V29" s="2"/>
+      <c r="W29" s="2"/>
     </row>
     <row r="30" spans="1:23" ht="15" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
@@ -2356,40 +2250,36 @@
       <c r="H30" t="s">
         <v>80</v>
       </c>
-      <c r="J30" s="2"/>
-      <c r="K30" s="2"/>
-      <c r="L30" s="2"/>
-      <c r="M30" s="2"/>
-      <c r="N30" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="O30" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="P30" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="Q30" s="2" t="s">
+      <c r="J30" s="2">
+        <v>60</v>
+      </c>
+      <c r="K30" s="2">
         <v>65</v>
       </c>
-      <c r="R30" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="S30" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="T30" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="U30" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="V30" s="2" t="s">
+      <c r="L30" s="2">
         <v>70</v>
       </c>
-      <c r="W30" s="2" t="s">
-        <v>51</v>
-      </c>
+      <c r="M30" s="2">
+        <v>75</v>
+      </c>
+      <c r="N30" s="2">
+        <v>85</v>
+      </c>
+      <c r="O30" s="2">
+        <v>95</v>
+      </c>
+      <c r="P30" s="2">
+        <v>110</v>
+      </c>
+      <c r="Q30" s="2">
+        <v>999</v>
+      </c>
+      <c r="R30" s="2"/>
+      <c r="S30" s="2"/>
+      <c r="T30" s="2"/>
+      <c r="U30" s="2"/>
+      <c r="V30" s="2"/>
+      <c r="W30" s="2"/>
     </row>
     <row r="31" spans="1:23" ht="15" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
@@ -2417,40 +2307,36 @@
       <c r="H31" t="s">
         <v>80</v>
       </c>
-      <c r="J31" s="2"/>
-      <c r="K31" s="2"/>
-      <c r="L31" s="2"/>
-      <c r="M31" s="2"/>
-      <c r="N31" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="O31" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="P31" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="Q31" s="2" t="s">
+      <c r="J31" s="2">
+        <v>60</v>
+      </c>
+      <c r="K31" s="2">
         <v>65</v>
       </c>
-      <c r="R31" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="S31" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="T31" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="U31" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="V31" s="2" t="s">
+      <c r="L31" s="2">
         <v>70</v>
       </c>
-      <c r="W31" s="2" t="s">
-        <v>51</v>
-      </c>
+      <c r="M31" s="2">
+        <v>75</v>
+      </c>
+      <c r="N31" s="2">
+        <v>85</v>
+      </c>
+      <c r="O31" s="2">
+        <v>95</v>
+      </c>
+      <c r="P31" s="2">
+        <v>110</v>
+      </c>
+      <c r="Q31" s="2">
+        <v>999</v>
+      </c>
+      <c r="R31" s="2"/>
+      <c r="S31" s="2"/>
+      <c r="T31" s="2"/>
+      <c r="U31" s="2"/>
+      <c r="V31" s="2"/>
+      <c r="W31" s="2"/>
     </row>
     <row r="32" spans="1:23" ht="15" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
@@ -2478,40 +2364,36 @@
       <c r="H32" t="s">
         <v>80</v>
       </c>
-      <c r="J32" s="2"/>
-      <c r="K32" s="2"/>
-      <c r="L32" s="2"/>
-      <c r="M32" s="2"/>
-      <c r="N32" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="O32" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="P32" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="Q32" s="2" t="s">
+      <c r="J32" s="2">
+        <v>60</v>
+      </c>
+      <c r="K32" s="2">
         <v>65</v>
       </c>
-      <c r="R32" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="S32" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="T32" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="U32" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="V32" s="2" t="s">
+      <c r="L32" s="2">
         <v>70</v>
       </c>
-      <c r="W32" s="2" t="s">
-        <v>51</v>
-      </c>
+      <c r="M32" s="2">
+        <v>75</v>
+      </c>
+      <c r="N32" s="2">
+        <v>85</v>
+      </c>
+      <c r="O32" s="2">
+        <v>95</v>
+      </c>
+      <c r="P32" s="2">
+        <v>110</v>
+      </c>
+      <c r="Q32" s="2">
+        <v>999</v>
+      </c>
+      <c r="R32" s="2"/>
+      <c r="S32" s="2"/>
+      <c r="T32" s="2"/>
+      <c r="U32" s="2"/>
+      <c r="V32" s="2"/>
+      <c r="W32" s="2"/>
     </row>
     <row r="33" spans="1:23" ht="15" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
@@ -2539,40 +2421,36 @@
       <c r="H33" t="s">
         <v>80</v>
       </c>
-      <c r="J33" s="2"/>
-      <c r="K33" s="2"/>
-      <c r="L33" s="2"/>
-      <c r="M33" s="2"/>
-      <c r="N33" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="O33" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="P33" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="Q33" s="2" t="s">
+      <c r="J33" s="2">
+        <v>60</v>
+      </c>
+      <c r="K33" s="2">
         <v>65</v>
       </c>
-      <c r="R33" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="S33" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="T33" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="U33" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="V33" s="2" t="s">
+      <c r="L33" s="2">
         <v>70</v>
       </c>
-      <c r="W33" s="2" t="s">
-        <v>51</v>
-      </c>
+      <c r="M33" s="2">
+        <v>75</v>
+      </c>
+      <c r="N33" s="2">
+        <v>85</v>
+      </c>
+      <c r="O33" s="2">
+        <v>95</v>
+      </c>
+      <c r="P33" s="2">
+        <v>110</v>
+      </c>
+      <c r="Q33" s="2">
+        <v>999</v>
+      </c>
+      <c r="R33" s="2"/>
+      <c r="S33" s="2"/>
+      <c r="T33" s="2"/>
+      <c r="U33" s="2"/>
+      <c r="V33" s="2"/>
+      <c r="W33" s="2"/>
     </row>
     <row r="34" spans="1:23" ht="15" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
@@ -2600,40 +2478,36 @@
       <c r="H34" t="s">
         <v>80</v>
       </c>
-      <c r="J34" s="2"/>
-      <c r="K34" s="2"/>
-      <c r="L34" s="2"/>
-      <c r="M34" s="2"/>
-      <c r="N34" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="O34" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="P34" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="Q34" s="2" t="s">
+      <c r="J34" s="2">
+        <v>60</v>
+      </c>
+      <c r="K34" s="2">
         <v>65</v>
       </c>
-      <c r="R34" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="S34" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="T34" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="U34" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="V34" s="2" t="s">
+      <c r="L34" s="2">
         <v>70</v>
       </c>
-      <c r="W34" s="2" t="s">
-        <v>51</v>
-      </c>
+      <c r="M34" s="2">
+        <v>75</v>
+      </c>
+      <c r="N34" s="2">
+        <v>85</v>
+      </c>
+      <c r="O34" s="2">
+        <v>95</v>
+      </c>
+      <c r="P34" s="2">
+        <v>110</v>
+      </c>
+      <c r="Q34" s="2">
+        <v>999</v>
+      </c>
+      <c r="R34" s="2"/>
+      <c r="S34" s="2"/>
+      <c r="T34" s="2"/>
+      <c r="U34" s="2"/>
+      <c r="V34" s="2"/>
+      <c r="W34" s="2"/>
     </row>
     <row r="35" spans="1:23" ht="15" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
@@ -2661,40 +2535,36 @@
       <c r="H35" t="s">
         <v>80</v>
       </c>
-      <c r="J35" s="2"/>
-      <c r="K35" s="2"/>
-      <c r="L35" s="2"/>
-      <c r="M35" s="2"/>
-      <c r="N35" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="O35" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="P35" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="Q35" s="2" t="s">
+      <c r="J35" s="2">
+        <v>60</v>
+      </c>
+      <c r="K35" s="2">
         <v>65</v>
       </c>
-      <c r="R35" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="S35" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="T35" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="U35" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="V35" s="2" t="s">
+      <c r="L35" s="2">
         <v>70</v>
       </c>
-      <c r="W35" s="2" t="s">
-        <v>51</v>
-      </c>
+      <c r="M35" s="2">
+        <v>75</v>
+      </c>
+      <c r="N35" s="2">
+        <v>85</v>
+      </c>
+      <c r="O35" s="2">
+        <v>95</v>
+      </c>
+      <c r="P35" s="2">
+        <v>110</v>
+      </c>
+      <c r="Q35" s="2">
+        <v>999</v>
+      </c>
+      <c r="R35" s="2"/>
+      <c r="S35" s="2"/>
+      <c r="T35" s="2"/>
+      <c r="U35" s="2"/>
+      <c r="V35" s="2"/>
+      <c r="W35" s="2"/>
     </row>
     <row r="36" spans="1:23" ht="15" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
@@ -2722,40 +2592,36 @@
       <c r="H36" t="s">
         <v>80</v>
       </c>
-      <c r="J36" s="2"/>
-      <c r="K36" s="2"/>
-      <c r="L36" s="2"/>
-      <c r="M36" s="2"/>
-      <c r="N36" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="O36" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="P36" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="Q36" s="2" t="s">
+      <c r="J36" s="2">
+        <v>60</v>
+      </c>
+      <c r="K36" s="2">
         <v>65</v>
       </c>
-      <c r="R36" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="S36" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="T36" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="U36" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="V36" s="2" t="s">
+      <c r="L36" s="2">
         <v>70</v>
       </c>
-      <c r="W36" s="2" t="s">
-        <v>51</v>
-      </c>
+      <c r="M36" s="2">
+        <v>75</v>
+      </c>
+      <c r="N36" s="2">
+        <v>85</v>
+      </c>
+      <c r="O36" s="2">
+        <v>95</v>
+      </c>
+      <c r="P36" s="2">
+        <v>110</v>
+      </c>
+      <c r="Q36" s="2">
+        <v>999</v>
+      </c>
+      <c r="R36" s="2"/>
+      <c r="S36" s="2"/>
+      <c r="T36" s="2"/>
+      <c r="U36" s="2"/>
+      <c r="V36" s="2"/>
+      <c r="W36" s="2"/>
     </row>
     <row r="37" spans="1:23" ht="15" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
@@ -2783,40 +2649,36 @@
       <c r="H37" t="s">
         <v>80</v>
       </c>
-      <c r="J37" s="2"/>
-      <c r="K37" s="2"/>
-      <c r="L37" s="2"/>
-      <c r="M37" s="2"/>
-      <c r="N37" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="O37" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="P37" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="Q37" s="2" t="s">
+      <c r="J37" s="2">
+        <v>60</v>
+      </c>
+      <c r="K37" s="2">
         <v>65</v>
       </c>
-      <c r="R37" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="S37" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="T37" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="U37" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="V37" s="2" t="s">
+      <c r="L37" s="2">
         <v>70</v>
       </c>
-      <c r="W37" s="2" t="s">
-        <v>51</v>
-      </c>
+      <c r="M37" s="2">
+        <v>75</v>
+      </c>
+      <c r="N37" s="2">
+        <v>85</v>
+      </c>
+      <c r="O37" s="2">
+        <v>95</v>
+      </c>
+      <c r="P37" s="2">
+        <v>110</v>
+      </c>
+      <c r="Q37" s="2">
+        <v>999</v>
+      </c>
+      <c r="R37" s="2"/>
+      <c r="S37" s="2"/>
+      <c r="T37" s="2"/>
+      <c r="U37" s="2"/>
+      <c r="V37" s="2"/>
+      <c r="W37" s="2"/>
     </row>
     <row r="38" spans="1:23" ht="15" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
@@ -2844,40 +2706,36 @@
       <c r="H38" t="s">
         <v>80</v>
       </c>
-      <c r="J38" s="2"/>
-      <c r="K38" s="2"/>
-      <c r="L38" s="2"/>
-      <c r="M38" s="2"/>
-      <c r="N38" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="O38" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="P38" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="Q38" s="2" t="s">
+      <c r="J38" s="2">
+        <v>60</v>
+      </c>
+      <c r="K38" s="2">
         <v>65</v>
       </c>
-      <c r="R38" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="S38" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="T38" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="U38" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="V38" s="2" t="s">
+      <c r="L38" s="2">
         <v>70</v>
       </c>
-      <c r="W38" s="2" t="s">
-        <v>51</v>
-      </c>
+      <c r="M38" s="2">
+        <v>75</v>
+      </c>
+      <c r="N38" s="2">
+        <v>85</v>
+      </c>
+      <c r="O38" s="2">
+        <v>95</v>
+      </c>
+      <c r="P38" s="2">
+        <v>110</v>
+      </c>
+      <c r="Q38" s="2">
+        <v>999</v>
+      </c>
+      <c r="R38" s="2"/>
+      <c r="S38" s="2"/>
+      <c r="T38" s="2"/>
+      <c r="U38" s="2"/>
+      <c r="V38" s="2"/>
+      <c r="W38" s="2"/>
     </row>
     <row r="39" spans="1:23" ht="15" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
@@ -2905,40 +2763,36 @@
       <c r="H39" t="s">
         <v>80</v>
       </c>
-      <c r="J39" s="2"/>
-      <c r="K39" s="2"/>
-      <c r="L39" s="2"/>
-      <c r="M39" s="2"/>
-      <c r="N39" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="O39" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="P39" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="Q39" s="2" t="s">
+      <c r="J39" s="2">
+        <v>60</v>
+      </c>
+      <c r="K39" s="2">
         <v>65</v>
       </c>
-      <c r="R39" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="S39" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="T39" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="U39" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="V39" s="2" t="s">
+      <c r="L39" s="2">
         <v>70</v>
       </c>
-      <c r="W39" s="2" t="s">
-        <v>51</v>
-      </c>
+      <c r="M39" s="2">
+        <v>75</v>
+      </c>
+      <c r="N39" s="2">
+        <v>85</v>
+      </c>
+      <c r="O39" s="2">
+        <v>95</v>
+      </c>
+      <c r="P39" s="2">
+        <v>110</v>
+      </c>
+      <c r="Q39" s="2">
+        <v>999</v>
+      </c>
+      <c r="R39" s="2"/>
+      <c r="S39" s="2"/>
+      <c r="T39" s="2"/>
+      <c r="U39" s="2"/>
+      <c r="V39" s="2"/>
+      <c r="W39" s="2"/>
     </row>
     <row r="40" spans="1:23" ht="15" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
@@ -2966,40 +2820,36 @@
       <c r="H40" t="s">
         <v>80</v>
       </c>
-      <c r="J40" s="2"/>
-      <c r="K40" s="2"/>
-      <c r="L40" s="2"/>
-      <c r="M40" s="2"/>
-      <c r="N40" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="O40" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="P40" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="Q40" s="2" t="s">
+      <c r="J40" s="2">
+        <v>60</v>
+      </c>
+      <c r="K40" s="2">
         <v>65</v>
       </c>
-      <c r="R40" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="S40" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="T40" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="U40" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="V40" s="2" t="s">
+      <c r="L40" s="2">
         <v>70</v>
       </c>
-      <c r="W40" s="2" t="s">
-        <v>51</v>
-      </c>
+      <c r="M40" s="2">
+        <v>75</v>
+      </c>
+      <c r="N40" s="2">
+        <v>85</v>
+      </c>
+      <c r="O40" s="2">
+        <v>95</v>
+      </c>
+      <c r="P40" s="2">
+        <v>110</v>
+      </c>
+      <c r="Q40" s="2">
+        <v>999</v>
+      </c>
+      <c r="R40" s="2"/>
+      <c r="S40" s="2"/>
+      <c r="T40" s="2"/>
+      <c r="U40" s="2"/>
+      <c r="V40" s="2"/>
+      <c r="W40" s="2"/>
     </row>
     <row r="41" spans="1:23" ht="15" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
@@ -3027,40 +2877,36 @@
       <c r="H41" t="s">
         <v>80</v>
       </c>
-      <c r="J41" s="2"/>
-      <c r="K41" s="2"/>
-      <c r="L41" s="2"/>
-      <c r="M41" s="2"/>
-      <c r="N41" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="O41" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="P41" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="Q41" s="2" t="s">
+      <c r="J41" s="2">
+        <v>60</v>
+      </c>
+      <c r="K41" s="2">
         <v>65</v>
       </c>
-      <c r="R41" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="S41" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="T41" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="U41" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="V41" s="2" t="s">
+      <c r="L41" s="2">
         <v>70</v>
       </c>
-      <c r="W41" s="2" t="s">
-        <v>51</v>
-      </c>
+      <c r="M41" s="2">
+        <v>75</v>
+      </c>
+      <c r="N41" s="2">
+        <v>85</v>
+      </c>
+      <c r="O41" s="2">
+        <v>95</v>
+      </c>
+      <c r="P41" s="2">
+        <v>110</v>
+      </c>
+      <c r="Q41" s="2">
+        <v>999</v>
+      </c>
+      <c r="R41" s="2"/>
+      <c r="S41" s="2"/>
+      <c r="T41" s="2"/>
+      <c r="U41" s="2"/>
+      <c r="V41" s="2"/>
+      <c r="W41" s="2"/>
     </row>
     <row r="42" spans="1:23" ht="15" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
@@ -3088,40 +2934,36 @@
       <c r="H42" t="s">
         <v>80</v>
       </c>
-      <c r="J42" s="2"/>
-      <c r="K42" s="2"/>
-      <c r="L42" s="2"/>
-      <c r="M42" s="2"/>
-      <c r="N42" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="O42" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="P42" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="Q42" s="2" t="s">
+      <c r="J42" s="2">
+        <v>60</v>
+      </c>
+      <c r="K42" s="2">
         <v>65</v>
       </c>
-      <c r="R42" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="S42" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="T42" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="U42" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="V42" s="2" t="s">
+      <c r="L42" s="2">
         <v>70</v>
       </c>
-      <c r="W42" s="2" t="s">
-        <v>51</v>
-      </c>
+      <c r="M42" s="2">
+        <v>75</v>
+      </c>
+      <c r="N42" s="2">
+        <v>85</v>
+      </c>
+      <c r="O42" s="2">
+        <v>95</v>
+      </c>
+      <c r="P42" s="2">
+        <v>110</v>
+      </c>
+      <c r="Q42" s="2">
+        <v>999</v>
+      </c>
+      <c r="R42" s="2"/>
+      <c r="S42" s="2"/>
+      <c r="T42" s="2"/>
+      <c r="U42" s="2"/>
+      <c r="V42" s="2"/>
+      <c r="W42" s="2"/>
     </row>
     <row r="43" spans="1:23" ht="15" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
@@ -3149,40 +2991,36 @@
       <c r="H43" t="s">
         <v>80</v>
       </c>
-      <c r="J43" s="2"/>
-      <c r="K43" s="2"/>
-      <c r="L43" s="2"/>
-      <c r="M43" s="2"/>
-      <c r="N43" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="O43" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="P43" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="Q43" s="2" t="s">
+      <c r="J43" s="2">
+        <v>60</v>
+      </c>
+      <c r="K43" s="2">
         <v>65</v>
       </c>
-      <c r="R43" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="S43" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="T43" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="U43" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="V43" s="2" t="s">
+      <c r="L43" s="2">
         <v>70</v>
       </c>
-      <c r="W43" s="2" t="s">
-        <v>51</v>
-      </c>
+      <c r="M43" s="2">
+        <v>75</v>
+      </c>
+      <c r="N43" s="2">
+        <v>85</v>
+      </c>
+      <c r="O43" s="2">
+        <v>95</v>
+      </c>
+      <c r="P43" s="2">
+        <v>110</v>
+      </c>
+      <c r="Q43" s="2">
+        <v>999</v>
+      </c>
+      <c r="R43" s="2"/>
+      <c r="S43" s="2"/>
+      <c r="T43" s="2"/>
+      <c r="U43" s="2"/>
+      <c r="V43" s="2"/>
+      <c r="W43" s="2"/>
     </row>
     <row r="44" spans="1:23" ht="15" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
@@ -3210,39 +3048,35 @@
       <c r="H44" t="s">
         <v>80</v>
       </c>
-      <c r="J44" s="2"/>
-      <c r="K44" s="2"/>
-      <c r="L44" s="2"/>
-      <c r="M44" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="N44" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="O44" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="P44" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="Q44" s="2" t="s">
+      <c r="J44" s="2">
+        <v>55</v>
+      </c>
+      <c r="K44" s="2">
+        <v>60</v>
+      </c>
+      <c r="L44" s="2">
         <v>65</v>
       </c>
-      <c r="R44" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="S44" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="T44" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="U44" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="V44" s="2" t="s">
-        <v>51</v>
-      </c>
+      <c r="M44" s="2">
+        <v>70</v>
+      </c>
+      <c r="N44" s="2">
+        <v>75</v>
+      </c>
+      <c r="O44" s="2">
+        <v>85</v>
+      </c>
+      <c r="P44" s="2">
+        <v>95</v>
+      </c>
+      <c r="Q44" s="2">
+        <v>999</v>
+      </c>
+      <c r="R44" s="2"/>
+      <c r="S44" s="2"/>
+      <c r="T44" s="2"/>
+      <c r="U44" s="2"/>
+      <c r="V44" s="2"/>
       <c r="W44" s="2"/>
     </row>
     <row r="45" spans="1:23" ht="15" x14ac:dyDescent="0.25">
@@ -3271,40 +3105,36 @@
       <c r="H45" t="s">
         <v>80</v>
       </c>
-      <c r="J45" s="2"/>
-      <c r="K45" s="2"/>
-      <c r="L45" s="2"/>
-      <c r="M45" s="2"/>
-      <c r="N45" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="O45" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="P45" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="Q45" s="2" t="s">
+      <c r="J45" s="2">
+        <v>60</v>
+      </c>
+      <c r="K45" s="2">
         <v>65</v>
       </c>
-      <c r="R45" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="S45" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="T45" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="U45" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="V45" s="2" t="s">
+      <c r="L45" s="2">
         <v>70</v>
       </c>
-      <c r="W45" s="2" t="s">
-        <v>51</v>
-      </c>
+      <c r="M45" s="2">
+        <v>75</v>
+      </c>
+      <c r="N45" s="2">
+        <v>85</v>
+      </c>
+      <c r="O45" s="2">
+        <v>95</v>
+      </c>
+      <c r="P45" s="2">
+        <v>110</v>
+      </c>
+      <c r="Q45" s="2">
+        <v>999</v>
+      </c>
+      <c r="R45" s="2"/>
+      <c r="S45" s="2"/>
+      <c r="T45" s="2"/>
+      <c r="U45" s="2"/>
+      <c r="V45" s="2"/>
+      <c r="W45" s="2"/>
     </row>
     <row r="46" spans="1:23" ht="15" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
@@ -3332,40 +3162,36 @@
       <c r="H46" t="s">
         <v>80</v>
       </c>
-      <c r="J46" s="2"/>
-      <c r="K46" s="2"/>
-      <c r="L46" s="2"/>
-      <c r="M46" s="2"/>
-      <c r="N46" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="O46" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="P46" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="Q46" s="2" t="s">
+      <c r="J46" s="2">
+        <v>60</v>
+      </c>
+      <c r="K46" s="2">
         <v>65</v>
       </c>
-      <c r="R46" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="S46" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="T46" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="U46" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="V46" s="2" t="s">
+      <c r="L46" s="2">
         <v>70</v>
       </c>
-      <c r="W46" s="2" t="s">
-        <v>51</v>
-      </c>
+      <c r="M46" s="2">
+        <v>75</v>
+      </c>
+      <c r="N46" s="2">
+        <v>85</v>
+      </c>
+      <c r="O46" s="2">
+        <v>95</v>
+      </c>
+      <c r="P46" s="2">
+        <v>110</v>
+      </c>
+      <c r="Q46" s="2">
+        <v>999</v>
+      </c>
+      <c r="R46" s="2"/>
+      <c r="S46" s="2"/>
+      <c r="T46" s="2"/>
+      <c r="U46" s="2"/>
+      <c r="V46" s="2"/>
+      <c r="W46" s="2"/>
     </row>
     <row r="47" spans="1:23" ht="15" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
@@ -3393,48 +3219,46 @@
       <c r="H47" t="s">
         <v>80</v>
       </c>
-      <c r="J47" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="K47" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="L47" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="M47" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="N47" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="O47" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="P47" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="Q47" s="2" t="s">
+      <c r="J47" s="2">
+        <v>35</v>
+      </c>
+      <c r="K47" s="2">
+        <v>40</v>
+      </c>
+      <c r="L47" s="2">
+        <v>45</v>
+      </c>
+      <c r="M47" s="2">
+        <v>50</v>
+      </c>
+      <c r="N47" s="2">
+        <v>55</v>
+      </c>
+      <c r="O47" s="2">
+        <v>60</v>
+      </c>
+      <c r="P47" s="2">
         <v>65</v>
       </c>
-      <c r="R47" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="S47" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="T47" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="U47" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="V47" s="2" t="s">
+      <c r="Q47" s="2">
         <v>70</v>
       </c>
-      <c r="W47" s="2" t="s">
-        <v>51</v>
-      </c>
+      <c r="R47" s="2">
+        <v>75</v>
+      </c>
+      <c r="S47" s="2">
+        <v>85</v>
+      </c>
+      <c r="T47" s="2">
+        <v>95</v>
+      </c>
+      <c r="U47" s="2">
+        <v>110</v>
+      </c>
+      <c r="V47" s="2">
+        <v>999</v>
+      </c>
+      <c r="W47" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>